<commit_message>
Refactor project structure and update API test cases; replace Preconditions with Hooks for better browser management and enhance dataset handling
</commit_message>
<xml_diff>
--- a/src/test/resources/api_data/datasets/dataset.xlsx
+++ b/src/test/resources/api_data/datasets/dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gmena\Java_DEMO\Herokuapp\src\test\resources\api_data\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9379EB0F-F391-41CB-9BB3-DA65EC89F7EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8948768-EB38-4DF0-92AE-119FD6C0693C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="57">
   <si>
     <t>firstName</t>
   </si>
@@ -78,13 +78,124 @@
     <t>jdoe@fake.com</t>
   </si>
   <si>
+    <t>8005555555</t>
+  </si>
+  <si>
+    <t>12345</t>
+  </si>
+  <si>
     <t>2022-11-12</t>
   </si>
   <si>
-    <t>8005555555</t>
-  </si>
-  <si>
-    <t>12345</t>
+    <t>_id</t>
+  </si>
+  <si>
+    <t>69cc0fb64938ae00154018aa</t>
+  </si>
+  <si>
+    <t>69cc0fb84938ae00154018ab</t>
+  </si>
+  <si>
+    <t>69cc1069220c4900159b090a</t>
+  </si>
+  <si>
+    <t>69cbf6f34938ae0015401839</t>
+  </si>
+  <si>
+    <t>69cbf70e4938ae001540183a</t>
+  </si>
+  <si>
+    <t>69cbf998220c4900159b0865</t>
+  </si>
+  <si>
+    <t>69cbfa6c220c4900159b086c</t>
+  </si>
+  <si>
+    <t>69cbfad24938ae0015401854</t>
+  </si>
+  <si>
+    <t>69cbfb3d4938ae001540185f</t>
+  </si>
+  <si>
+    <t>69cbfb3e220c4900159b087f</t>
+  </si>
+  <si>
+    <t>69cc05314938ae001540187d</t>
+  </si>
+  <si>
+    <t>69cc05324938ae001540187f</t>
+  </si>
+  <si>
+    <t>69cc059c4938ae0015401880</t>
+  </si>
+  <si>
+    <t>69cc059d220c4900159b08a1</t>
+  </si>
+  <si>
+    <t>69cc0a0c4938ae0015401889</t>
+  </si>
+  <si>
+    <t>69cc0a0d220c4900159b08aa</t>
+  </si>
+  <si>
+    <t>69cc0a5b4938ae001540188b</t>
+  </si>
+  <si>
+    <t>69cc0a5c220c4900159b08ad</t>
+  </si>
+  <si>
+    <t>69cc0b4c220c4900159b08af</t>
+  </si>
+  <si>
+    <t>69cc0b4e4938ae001540188d</t>
+  </si>
+  <si>
+    <t>69cc0bf0220c4900159b08b3</t>
+  </si>
+  <si>
+    <t>69cc0bf14938ae001540188f</t>
+  </si>
+  <si>
+    <t>69cc0c6c4938ae0015401890</t>
+  </si>
+  <si>
+    <t>69cc0c6d220c4900159b08b7</t>
+  </si>
+  <si>
+    <t>69cc0cd64938ae0015401893</t>
+  </si>
+  <si>
+    <t>69cc0cd8220c4900159b08b9</t>
+  </si>
+  <si>
+    <t>69cc0dec220c4900159b08c1</t>
+  </si>
+  <si>
+    <t>69cc0ded4938ae001540189c</t>
+  </si>
+  <si>
+    <t>69cc0e30220c4900159b08c4</t>
+  </si>
+  <si>
+    <t>69cc0e31220c4900159b08c6</t>
+  </si>
+  <si>
+    <t>69cc0e53220c4900159b08c8</t>
+  </si>
+  <si>
+    <t>69cc0e544938ae00154018a0</t>
+  </si>
+  <si>
+    <t>69cc0ec44938ae00154018a4</t>
+  </si>
+  <si>
+    <t>69cc0ec5220c4900159b08cd</t>
+  </si>
+  <si>
+    <t>69cc0f12220c4900159b08ce</t>
+  </si>
+  <si>
+    <t>69cc0f13220c4900159b08d0</t>
   </si>
 </sst>
 </file>
@@ -426,65 +537,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="12" width="24.140625" customWidth="1"/>
+    <col min="2" max="13" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
       </c>
       <c r="G2" t="s">
         <v>12</v>
@@ -492,14 +606,210 @@
       <c r="H2" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="J2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" t="s">
-        <v>14</v>
+      <c r="E3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add user management features and API error validation
- Created JSON template for adding a user with email, password, first name, and last name.
- Added error messages for various validation scenarios in the properties file.
- Implemented smoke and end-to-end test cases for web application features including user signup and login.
- Developed API test cases for adding, retrieving, updating, and deleting contacts, including error validation for missing and incorrect fields.
- Added scenarios for testing user deletion and ensuring proper cleanup after tests.
</commit_message>
<xml_diff>
--- a/src/test/resources/api_data/datasets/dataset.xlsx
+++ b/src/test/resources/api_data/datasets/dataset.xlsx
@@ -3,21 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gmena\Java_DEMO\Herokuapp\src\test\resources\api_data\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8948768-EB38-4DF0-92AE-119FD6C0693C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967CA68B-6E42-4603-BD14-91330C19F0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="61">
   <si>
     <t>firstName</t>
   </si>
@@ -90,118 +90,131 @@
     <t>_id</t>
   </si>
   <si>
-    <t>69cc0fb64938ae00154018aa</t>
-  </si>
-  <si>
-    <t>69cc0fb84938ae00154018ab</t>
-  </si>
-  <si>
-    <t>69cc1069220c4900159b090a</t>
-  </si>
-  <si>
-    <t>69cbf6f34938ae0015401839</t>
-  </si>
-  <si>
-    <t>69cbf70e4938ae001540183a</t>
-  </si>
-  <si>
-    <t>69cbf998220c4900159b0865</t>
-  </si>
-  <si>
-    <t>69cbfa6c220c4900159b086c</t>
-  </si>
-  <si>
-    <t>69cbfad24938ae0015401854</t>
-  </si>
-  <si>
-    <t>69cbfb3d4938ae001540185f</t>
-  </si>
-  <si>
-    <t>69cbfb3e220c4900159b087f</t>
-  </si>
-  <si>
-    <t>69cc05314938ae001540187d</t>
-  </si>
-  <si>
-    <t>69cc05324938ae001540187f</t>
-  </si>
-  <si>
-    <t>69cc059c4938ae0015401880</t>
-  </si>
-  <si>
-    <t>69cc059d220c4900159b08a1</t>
-  </si>
-  <si>
-    <t>69cc0a0c4938ae0015401889</t>
-  </si>
-  <si>
-    <t>69cc0a0d220c4900159b08aa</t>
-  </si>
-  <si>
-    <t>69cc0a5b4938ae001540188b</t>
-  </si>
-  <si>
-    <t>69cc0a5c220c4900159b08ad</t>
-  </si>
-  <si>
-    <t>69cc0b4c220c4900159b08af</t>
-  </si>
-  <si>
-    <t>69cc0b4e4938ae001540188d</t>
-  </si>
-  <si>
-    <t>69cc0bf0220c4900159b08b3</t>
-  </si>
-  <si>
-    <t>69cc0bf14938ae001540188f</t>
-  </si>
-  <si>
-    <t>69cc0c6c4938ae0015401890</t>
-  </si>
-  <si>
-    <t>69cc0c6d220c4900159b08b7</t>
-  </si>
-  <si>
-    <t>69cc0cd64938ae0015401893</t>
-  </si>
-  <si>
-    <t>69cc0cd8220c4900159b08b9</t>
-  </si>
-  <si>
-    <t>69cc0dec220c4900159b08c1</t>
-  </si>
-  <si>
-    <t>69cc0ded4938ae001540189c</t>
-  </si>
-  <si>
-    <t>69cc0e30220c4900159b08c4</t>
-  </si>
-  <si>
-    <t>69cc0e31220c4900159b08c6</t>
-  </si>
-  <si>
-    <t>69cc0e53220c4900159b08c8</t>
-  </si>
-  <si>
-    <t>69cc0e544938ae00154018a0</t>
-  </si>
-  <si>
-    <t>69cc0ec44938ae00154018a4</t>
-  </si>
-  <si>
-    <t>69cc0ec5220c4900159b08cd</t>
-  </si>
-  <si>
-    <t>69cc0f12220c4900159b08ce</t>
-  </si>
-  <si>
-    <t>69cc0f13220c4900159b08d0</t>
+    <t>Mark</t>
+  </si>
+  <si>
+    <t>O'Connor</t>
+  </si>
+  <si>
+    <t>69ccbe8fe174bc00158a265</t>
+  </si>
+  <si>
+    <t>69cce10d23b8a000159cb132</t>
+  </si>
+  <si>
+    <t>69cce745e174bc00158a2794</t>
+  </si>
+  <si>
+    <t>69cce82523b8a000159cb15d</t>
+  </si>
+  <si>
+    <t>69cce827e174bc00158a2799</t>
+  </si>
+  <si>
+    <t>69cce82923b8a000159cb160</t>
+  </si>
+  <si>
+    <t>69cceee423b8a000159cb17d</t>
+  </si>
+  <si>
+    <t>69ccf11de174bc00158a27b6</t>
+  </si>
+  <si>
+    <t>69ccf12023b8a000159cb17e</t>
+  </si>
+  <si>
+    <t>69ccf14223b8a000159cb17f</t>
+  </si>
+  <si>
+    <t>69ccf145e174bc00158a27ba</t>
+  </si>
+  <si>
+    <t>69ccf2c1e174bc00158a27bb</t>
+  </si>
+  <si>
+    <t>69ccf2c4e174bc00158a27bc</t>
+  </si>
+  <si>
+    <t>69ccf2f3e174bc00158a27bd</t>
+  </si>
+  <si>
+    <t>69ccf2f6e174bc00158a27be</t>
+  </si>
+  <si>
+    <t>69ccf36023b8a000159cb186</t>
+  </si>
+  <si>
+    <t>69ccf363e174bc00158a27c0</t>
+  </si>
+  <si>
+    <t>69ccf3e923b8a000159cb18c</t>
+  </si>
+  <si>
+    <t>Bob</t>
+  </si>
+  <si>
+    <t>69ccf440e174bc00158a2805</t>
+  </si>
+  <si>
+    <t>69ccf44323b8a000159cb1bd</t>
+  </si>
+  <si>
+    <t>69ccf445e174bc00158a2807</t>
+  </si>
+  <si>
+    <t>69ccf44923b8a000159cb1c0</t>
+  </si>
+  <si>
+    <t>69ccf44c23b8a000159cb1c2</t>
+  </si>
+  <si>
+    <t>69ccfd43e174bc00158a284e</t>
+  </si>
+  <si>
+    <t>69ccfd79e174bc00158a2853</t>
+  </si>
+  <si>
+    <t>69ccfe69e174bc00158a285e</t>
+  </si>
+  <si>
+    <t>69ccfec023b8a000159cb23c</t>
+  </si>
+  <si>
+    <t>69ccfec2e174bc00158a289e</t>
+  </si>
+  <si>
+    <t>69ccfec5e174bc00158a289f</t>
+  </si>
+  <si>
+    <t>69ccfec823b8a000159cb23f</t>
+  </si>
+  <si>
+    <t>69ccfecb23b8a000159cb240</t>
+  </si>
+  <si>
+    <t>69ccff6823b8a000159cb254</t>
+  </si>
+  <si>
+    <t>69ccffbe23b8a000159cb281</t>
+  </si>
+  <si>
+    <t>69ccffc023b8a000159cb282</t>
+  </si>
+  <si>
+    <t>69ccffc323b8a000159cb284</t>
+  </si>
+  <si>
+    <t>69ccffc723b8a000159cb285</t>
+  </si>
+  <si>
+    <t>69ccffc923b8a000159cb287</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -537,10 +550,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="13" width="24.140625" customWidth="1"/>
+    <col min="2" max="13" customWidth="true" width="24.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -582,14 +595,14 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
+      <c r="A2" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>22</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>19</v>
@@ -600,33 +613,33 @@
       <c r="F2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>12</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="A3" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="0">
         <v>11</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -640,176 +653,6 @@
       </c>
       <c r="J3" s="1" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance documentation and improve error handling across various classes
- Added Javadoc comments to POM classes (POM_ContactList, POM_Login, POM_SignUp) to describe methods and their functionality.
- Improved error message clarity in the Endpoint class.
- Updated UtilityReader class with additional methods for reading JSON and writing values to Excel datasets.
- Enhanced REST and RestOperations classes with detailed method descriptions.
- Added comments to Hooks class for better understanding of browser session management.
- Documented step definitions in ApiSteps and WebSteps for clarity on their purpose and parameters.
</commit_message>
<xml_diff>
--- a/src/test/resources/api_data/datasets/dataset.xlsx
+++ b/src/test/resources/api_data/datasets/dataset.xlsx
@@ -3,21 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gmena\Java_DEMO\Herokuapp\src\test\resources\api_data\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967CA68B-6E42-4603-BD14-91330C19F0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FC0295-544F-4A74-B20C-C45BCAD5BC93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
   <si>
     <t>firstName</t>
   </si>
@@ -94,127 +94,12 @@
   </si>
   <si>
     <t>O'Connor</t>
-  </si>
-  <si>
-    <t>69ccbe8fe174bc00158a265</t>
-  </si>
-  <si>
-    <t>69cce10d23b8a000159cb132</t>
-  </si>
-  <si>
-    <t>69cce745e174bc00158a2794</t>
-  </si>
-  <si>
-    <t>69cce82523b8a000159cb15d</t>
-  </si>
-  <si>
-    <t>69cce827e174bc00158a2799</t>
-  </si>
-  <si>
-    <t>69cce82923b8a000159cb160</t>
-  </si>
-  <si>
-    <t>69cceee423b8a000159cb17d</t>
-  </si>
-  <si>
-    <t>69ccf11de174bc00158a27b6</t>
-  </si>
-  <si>
-    <t>69ccf12023b8a000159cb17e</t>
-  </si>
-  <si>
-    <t>69ccf14223b8a000159cb17f</t>
-  </si>
-  <si>
-    <t>69ccf145e174bc00158a27ba</t>
-  </si>
-  <si>
-    <t>69ccf2c1e174bc00158a27bb</t>
-  </si>
-  <si>
-    <t>69ccf2c4e174bc00158a27bc</t>
-  </si>
-  <si>
-    <t>69ccf2f3e174bc00158a27bd</t>
-  </si>
-  <si>
-    <t>69ccf2f6e174bc00158a27be</t>
-  </si>
-  <si>
-    <t>69ccf36023b8a000159cb186</t>
-  </si>
-  <si>
-    <t>69ccf363e174bc00158a27c0</t>
-  </si>
-  <si>
-    <t>69ccf3e923b8a000159cb18c</t>
-  </si>
-  <si>
-    <t>Bob</t>
-  </si>
-  <si>
-    <t>69ccf440e174bc00158a2805</t>
-  </si>
-  <si>
-    <t>69ccf44323b8a000159cb1bd</t>
-  </si>
-  <si>
-    <t>69ccf445e174bc00158a2807</t>
-  </si>
-  <si>
-    <t>69ccf44923b8a000159cb1c0</t>
-  </si>
-  <si>
-    <t>69ccf44c23b8a000159cb1c2</t>
-  </si>
-  <si>
-    <t>69ccfd43e174bc00158a284e</t>
-  </si>
-  <si>
-    <t>69ccfd79e174bc00158a2853</t>
-  </si>
-  <si>
-    <t>69ccfe69e174bc00158a285e</t>
-  </si>
-  <si>
-    <t>69ccfec023b8a000159cb23c</t>
-  </si>
-  <si>
-    <t>69ccfec2e174bc00158a289e</t>
-  </si>
-  <si>
-    <t>69ccfec5e174bc00158a289f</t>
-  </si>
-  <si>
-    <t>69ccfec823b8a000159cb23f</t>
-  </si>
-  <si>
-    <t>69ccfecb23b8a000159cb240</t>
-  </si>
-  <si>
-    <t>69ccff6823b8a000159cb254</t>
-  </si>
-  <si>
-    <t>69ccffbe23b8a000159cb281</t>
-  </si>
-  <si>
-    <t>69ccffc023b8a000159cb282</t>
-  </si>
-  <si>
-    <t>69ccffc323b8a000159cb284</t>
-  </si>
-  <si>
-    <t>69ccffc723b8a000159cb285</t>
-  </si>
-  <si>
-    <t>69ccffc923b8a000159cb287</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -553,7 +438,7 @@
   <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="13" customWidth="true" width="24.140625"/>
+    <col min="2" max="13" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -595,13 +480,10 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
-        <v>60</v>
-      </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>21</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>22</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -613,33 +495,30 @@
       <c r="F2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="H2" t="s" s="0">
+      <c r="H2" t="s">
         <v>12</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>12</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K2" t="s" s="0">
+      <c r="K2" t="s">
         <v>13</v>
       </c>
-      <c r="L2" t="s" s="0">
+      <c r="L2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="1" t="s">

</xml_diff>